<commit_message>
cambio deprecvio de perfumina
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\OneDrive\Escritorio\bio-quim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BDB10C8-B1F0-4AAE-B09A-9D0B88D2065A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{164082F8-ABBD-46E6-8680-4100532FE312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -984,7 +984,7 @@
         <v>55</v>
       </c>
       <c r="D16">
-        <v>1900</v>
+        <v>9500</v>
       </c>
       <c r="E16" t="s">
         <v>64</v>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="D27">
         <f t="shared" si="0"/>
-        <v>9500</v>
+        <v>47500</v>
       </c>
       <c r="E27" t="s">
         <v>67</v>

</xml_diff>